<commit_message>
Preparation publication release 407 0ee7b72a25f29f75a692946a54d016f261abf699
</commit_message>
<xml_diff>
--- a/361-preparation-publication-release-407/ig/CodeSystem-input-task-sdo-codesystem.xlsx
+++ b/361-preparation-publication-release-407/ig/CodeSystem-input-task-sdo-codesystem.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>4.0.6</t>
+    <t>4.0.7</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-26T16:13:39+00:00</t>
+    <t>2026-06-26T16:22:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>